<commit_message>
Primo upload referti per validazione FSE 2026-05-04
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#FACTORYSOFTXX/GalassiaNG/1.0/accreditamento-checklist_V9.0.0.xlsx
+++ b/GATEWAY/A1#111#FACTORYSOFTXX/GalassiaNG/1.0/accreditamento-checklist_V9.0.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="-15" windowWidth="38460" windowHeight="14460" activeTab="2"/>
+    <workbookView xWindow="450" yWindow="7230" windowWidth="38460" windowHeight="10560" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -16,6 +16,7 @@
   </sheets>
   <externalReferences>
     <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Summary!$A$1:$G$10</definedName>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="636">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1682" uniqueCount="649">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -2400,14 +2401,53 @@
     <t>Errore timeout connessione, impossibile contattare il GW FSE</t>
   </si>
   <si>
-    <t>L’errore viene segnalato all’utente e nei log testuali dell’applicativo. Il medico o il back-office possono effettuare l’invio del documento premendo nuovamente, nella UI, l’apposito pulsante “Valida documento FSE”</t>
-  </si>
-  <si>
     <t xml:space="preserve">L’applicativo non gestisce tutti i campi richiesti dal test. Ma è limitato ad un set di tag, completo, di quelli ritenuti OBBLIGATORI.
 </t>
   </si>
   <si>
-    <t>confidentialityCode fisso a N</t>
+    <t>2.16.840.1.113883.2.9.99.9.2bdd653066d5b0a7e627f311b7c1ffa6d22c8ddbbd5466526e605f70db07e347.e6aa62d992^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t>8b28a77786a391f7b0aa77ea2daaf7bc</t>
+  </si>
+  <si>
+    <t>34b56d40afa69f97cb6336047e245698</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.99.9.2b60573de8ae21c79537d64043bf2a967eb53dfa369df02ddfab93939873519d.444adf945e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Errore durante la richiesta di validazione: campo token JWT non valido.  Il campo purpose_of_use non è valorizzato </t>
+  </si>
+  <si>
+    <t>L’errore viene segnalato all’utente che lo segnalerà all’assistenza tecnica di Factorysoft. Una volta trovata e applicata la soluzione, l’utente finale (medico) o il back-office potrà effettuare l’invio del documento.</t>
+  </si>
+  <si>
+    <t>add68eb132bddb7a5e37960716a3c47b</t>
+  </si>
+  <si>
+    <t>1614398472b6c4962032781c7452c3ea</t>
+  </si>
+  <si>
+    <t>a1d1885719ca3c1b11e01b706b81e389</t>
+  </si>
+  <si>
+    <t>a7ed534c2b571d3626cd881497eb1fe2</t>
+  </si>
+  <si>
+    <t>confidentialityCode impostato di default a N e modificato solo al bisogno  tramite selezione da un set di valori ammessi</t>
+  </si>
+  <si>
+    <t>051804937bd11a9f580798f430cd26f2</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.99.9.ee2a07d80a6fcac38a12465dddcd02ea18378dc059fbf28ba668345a5034b91f.454ab6b6e0</t>
+  </si>
+  <si>
+    <t>Errore vocabolario.","detail":"Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: 666.6]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Errore nel CDA. Errore terminologico. Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: 666.6] </t>
   </si>
 </sst>
 </file>
@@ -2595,12 +2635,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -2608,6 +2642,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3009,7 +3049,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3202,13 +3242,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -3222,10 +3256,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3238,6 +3272,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3261,6 +3301,18 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -3358,6 +3410,29 @@
       <sheetData sheetId="3"/>
       <sheetData sheetId="4" refreshError="1"/>
       <sheetData sheetId="5" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Istruzioni Compilazione"/>
+      <sheetName val="Prerequisiti"/>
+      <sheetName val="TestCases"/>
+      <sheetName val="LISTA VALORI"/>
+      <sheetName val="Summary"/>
+      <sheetName val="Sheet1"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -3740,7 +3815,7 @@
   <cols>
     <col min="1" max="1" width="11.42578125" customWidth="1"/>
     <col min="2" max="2" width="46.85546875" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" style="77" customWidth="1"/>
+    <col min="3" max="3" width="20.140625" style="75" customWidth="1"/>
     <col min="4" max="4" width="63.85546875" customWidth="1"/>
     <col min="5" max="5" width="104.85546875" customWidth="1"/>
     <col min="6" max="9" width="33.140625" customWidth="1"/>
@@ -3754,7 +3829,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="16.5" customHeight="1">
-      <c r="C1" s="75"/>
+      <c r="C1" s="73"/>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
@@ -3884,7 +3959,7 @@
     <row r="6" spans="1:23" ht="16.5" customHeight="1">
       <c r="A6" s="86"/>
       <c r="B6" s="87"/>
-      <c r="C6" s="76"/>
+      <c r="C6" s="74"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -3907,7 +3982,7 @@
     <row r="7" spans="1:23" ht="16.5" customHeight="1">
       <c r="A7" s="10"/>
       <c r="B7" s="10"/>
-      <c r="C7" s="76"/>
+      <c r="C7" s="74"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -3954,7 +4029,7 @@
       <c r="B9" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="78" t="s">
+      <c r="C9" s="76" t="s">
         <v>21</v>
       </c>
       <c r="D9" s="17" t="s">
@@ -4166,14 +4241,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="14" spans="1:23" ht="27" customHeight="1" thickBot="1">
       <c r="A14" s="29">
         <v>31</v>
       </c>
       <c r="B14" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="79" t="s">
+      <c r="C14" s="78" t="s">
         <v>54</v>
       </c>
       <c r="D14" s="29" t="s">
@@ -4182,20 +4257,40 @@
       <c r="E14" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="F14" s="31"/>
+      <c r="F14" s="31">
+        <v>46145</v>
+      </c>
       <c r="G14" s="31"/>
-      <c r="H14" s="31"/>
+      <c r="H14" s="31" t="s">
+        <v>640</v>
+      </c>
       <c r="I14" s="36"/>
-      <c r="J14" s="32"/>
+      <c r="J14" s="80" t="s">
+        <v>75</v>
+      </c>
       <c r="K14" s="32"/>
       <c r="L14" s="32"/>
-      <c r="M14" s="32"/>
-      <c r="N14" s="32"/>
-      <c r="O14" s="32"/>
-      <c r="P14" s="32"/>
-      <c r="Q14" s="32"/>
-      <c r="R14" s="32"/>
-      <c r="S14" s="32"/>
+      <c r="M14" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="N14" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="O14" s="71" t="s">
+        <v>638</v>
+      </c>
+      <c r="P14" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="Q14" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="R14" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="S14" s="84" t="s">
+        <v>639</v>
+      </c>
       <c r="T14" s="32"/>
       <c r="U14" s="33"/>
       <c r="V14" s="34"/>
@@ -4203,7 +4298,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="15" spans="1:23" ht="27" customHeight="1" thickBot="1">
       <c r="A15" s="29">
         <v>32</v>
       </c>
@@ -4219,20 +4314,40 @@
       <c r="E15" s="37" t="s">
         <v>48</v>
       </c>
-      <c r="F15" s="31"/>
+      <c r="F15" s="31">
+        <v>46145</v>
+      </c>
       <c r="G15" s="31"/>
-      <c r="H15" s="31"/>
+      <c r="H15" s="31" t="s">
+        <v>641</v>
+      </c>
       <c r="I15" s="36"/>
-      <c r="J15" s="32"/>
-      <c r="K15" s="32"/>
-      <c r="L15" s="32"/>
-      <c r="M15" s="32"/>
-      <c r="N15" s="32"/>
-      <c r="O15" s="32"/>
-      <c r="P15" s="32"/>
-      <c r="Q15" s="32"/>
-      <c r="R15" s="32"/>
-      <c r="S15" s="32"/>
+      <c r="J15" s="80" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="80"/>
+      <c r="L15" s="80"/>
+      <c r="M15" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="N15" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="O15" s="71" t="s">
+        <v>638</v>
+      </c>
+      <c r="P15" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="Q15" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="R15" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="S15" s="84" t="s">
+        <v>639</v>
+      </c>
       <c r="T15" s="32"/>
       <c r="U15" s="33"/>
       <c r="V15" s="34"/>
@@ -4462,14 +4577,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="22" spans="1:23" ht="27" customHeight="1" thickBot="1">
       <c r="A22" s="29">
         <v>39</v>
       </c>
       <c r="B22" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="79" t="s">
+      <c r="C22" s="78" t="s">
         <v>54</v>
       </c>
       <c r="D22" s="29" t="s">
@@ -4478,20 +4593,40 @@
       <c r="E22" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="F22" s="31"/>
+      <c r="F22" s="31">
+        <v>46145</v>
+      </c>
       <c r="G22" s="31"/>
-      <c r="H22" s="31"/>
+      <c r="H22" s="31" t="s">
+        <v>642</v>
+      </c>
       <c r="I22" s="36"/>
-      <c r="J22" s="32"/>
+      <c r="J22" s="80" t="s">
+        <v>75</v>
+      </c>
       <c r="K22" s="32"/>
       <c r="L22" s="32"/>
-      <c r="M22" s="32"/>
-      <c r="N22" s="32"/>
-      <c r="O22" s="32"/>
-      <c r="P22" s="32"/>
-      <c r="Q22" s="32"/>
-      <c r="R22" s="32"/>
-      <c r="S22" s="32"/>
+      <c r="M22" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="N22" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="O22" s="71" t="s">
+        <v>638</v>
+      </c>
+      <c r="P22" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="Q22" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="R22" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="S22" s="84" t="s">
+        <v>639</v>
+      </c>
       <c r="T22" s="32"/>
       <c r="U22" s="33"/>
       <c r="V22" s="34"/>
@@ -4499,7 +4634,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="23" spans="1:23" ht="27" customHeight="1" thickBot="1">
       <c r="A23" s="29">
         <v>40</v>
       </c>
@@ -4515,20 +4650,40 @@
       <c r="E23" s="37" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="31"/>
+      <c r="F23" s="31">
+        <v>46145</v>
+      </c>
       <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
+      <c r="H23" s="31" t="s">
+        <v>643</v>
+      </c>
       <c r="I23" s="36"/>
-      <c r="J23" s="32"/>
-      <c r="K23" s="32"/>
-      <c r="L23" s="32"/>
-      <c r="M23" s="32"/>
-      <c r="N23" s="32"/>
-      <c r="O23" s="32"/>
-      <c r="P23" s="32"/>
-      <c r="Q23" s="32"/>
-      <c r="R23" s="32"/>
-      <c r="S23" s="32"/>
+      <c r="J23" s="80" t="s">
+        <v>75</v>
+      </c>
+      <c r="K23" s="80"/>
+      <c r="L23" s="80"/>
+      <c r="M23" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="N23" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="O23" s="71" t="s">
+        <v>638</v>
+      </c>
+      <c r="P23" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="Q23" s="71" t="s">
+        <v>541</v>
+      </c>
+      <c r="R23" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="S23" s="84" t="s">
+        <v>639</v>
+      </c>
       <c r="T23" s="32"/>
       <c r="U23" s="33"/>
       <c r="V23" s="34"/>
@@ -4764,14 +4919,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="97.5" customHeight="1" thickBot="1">
+    <row r="30" spans="1:23" ht="27.75" customHeight="1" thickBot="1">
       <c r="A30" s="29">
         <v>47</v>
       </c>
       <c r="B30" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="79" t="s">
+      <c r="C30" s="78" t="s">
         <v>54</v>
       </c>
       <c r="D30" s="29" t="s">
@@ -4807,8 +4962,8 @@
       <c r="R30" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="S30" s="72" t="s">
-        <v>633</v>
+      <c r="S30" s="84" t="s">
+        <v>639</v>
       </c>
       <c r="T30" s="32"/>
       <c r="U30" s="33" t="s">
@@ -4819,7 +4974,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="101.25" customHeight="1" thickBot="1">
+    <row r="31" spans="1:23" ht="27.75" customHeight="1" thickBot="1">
       <c r="A31" s="29">
         <v>48</v>
       </c>
@@ -4835,9 +4990,7 @@
       <c r="E31" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="F31" s="31">
-        <v>46122</v>
-      </c>
+      <c r="F31" s="31"/>
       <c r="G31" s="31"/>
       <c r="H31" s="31"/>
       <c r="I31" s="36"/>
@@ -4864,8 +5017,8 @@
       <c r="R31" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="S31" s="72" t="s">
-        <v>633</v>
+      <c r="S31" s="84" t="s">
+        <v>639</v>
       </c>
       <c r="T31" s="32"/>
       <c r="U31" s="33" t="s">
@@ -5764,7 +5917,7 @@
       <c r="J55" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K55" s="82" t="s">
+      <c r="K55" s="80" t="s">
         <v>504</v>
       </c>
       <c r="L55" s="32"/>
@@ -5805,7 +5958,7 @@
       <c r="J56" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K56" s="73" t="s">
+      <c r="K56" s="72" t="s">
         <v>503</v>
       </c>
       <c r="L56" s="32"/>
@@ -5830,7 +5983,7 @@
       <c r="B57" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C57" s="83" t="s">
+      <c r="C57" s="81" t="s">
         <v>54</v>
       </c>
       <c r="D57" s="29" t="s">
@@ -5846,7 +5999,7 @@
       <c r="J57" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K57" s="82" t="s">
+      <c r="K57" s="80" t="s">
         <v>504</v>
       </c>
       <c r="L57" s="32"/>
@@ -5871,7 +6024,7 @@
       <c r="B58" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C58" s="83" t="s">
+      <c r="C58" s="81" t="s">
         <v>54</v>
       </c>
       <c r="D58" s="29" t="s">
@@ -5912,7 +6065,7 @@
       <c r="B59" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C59" s="83" t="s">
+      <c r="C59" s="81" t="s">
         <v>54</v>
       </c>
       <c r="D59" s="29" t="s">
@@ -5949,7 +6102,7 @@
       <c r="B60" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C60" s="83" t="s">
+      <c r="C60" s="81" t="s">
         <v>54</v>
       </c>
       <c r="D60" s="29" t="s">
@@ -5990,7 +6143,7 @@
       <c r="B61" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C61" s="79" t="s">
+      <c r="C61" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D61" s="29" t="s">
@@ -6003,14 +6156,14 @@
       <c r="G61" s="31"/>
       <c r="H61" s="31"/>
       <c r="I61" s="36"/>
-      <c r="J61" s="82" t="s">
+      <c r="J61" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K61" s="82" t="s">
+      <c r="K61" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L61" s="82" t="s">
-        <v>634</v>
+      <c r="L61" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M61" s="32"/>
       <c r="N61" s="32"/>
@@ -6033,7 +6186,7 @@
       <c r="B62" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C62" s="79" t="s">
+      <c r="C62" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D62" s="29" t="s">
@@ -6046,14 +6199,14 @@
       <c r="G62" s="31"/>
       <c r="H62" s="31"/>
       <c r="I62" s="36"/>
-      <c r="J62" s="82" t="s">
+      <c r="J62" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K62" s="82" t="s">
+      <c r="K62" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L62" s="82" t="s">
-        <v>634</v>
+      <c r="L62" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M62" s="32"/>
       <c r="N62" s="32"/>
@@ -6076,7 +6229,7 @@
       <c r="B63" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C63" s="79" t="s">
+      <c r="C63" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D63" s="29" t="s">
@@ -6089,14 +6242,14 @@
       <c r="G63" s="31"/>
       <c r="H63" s="31"/>
       <c r="I63" s="36"/>
-      <c r="J63" s="82" t="s">
+      <c r="J63" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K63" s="82" t="s">
+      <c r="K63" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L63" s="82" t="s">
-        <v>634</v>
+      <c r="L63" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M63" s="32"/>
       <c r="N63" s="32"/>
@@ -6119,7 +6272,7 @@
       <c r="B64" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C64" s="79" t="s">
+      <c r="C64" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D64" s="29" t="s">
@@ -6132,14 +6285,14 @@
       <c r="G64" s="31"/>
       <c r="H64" s="31"/>
       <c r="I64" s="36"/>
-      <c r="J64" s="82" t="s">
+      <c r="J64" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K64" s="82" t="s">
+      <c r="K64" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L64" s="82" t="s">
-        <v>634</v>
+      <c r="L64" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M64" s="32"/>
       <c r="N64" s="32"/>
@@ -6162,7 +6315,7 @@
       <c r="B65" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C65" s="79" t="s">
+      <c r="C65" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D65" s="29" t="s">
@@ -6175,14 +6328,14 @@
       <c r="G65" s="31"/>
       <c r="H65" s="31"/>
       <c r="I65" s="36"/>
-      <c r="J65" s="82" t="s">
+      <c r="J65" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K65" s="82" t="s">
+      <c r="K65" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L65" s="82" t="s">
-        <v>634</v>
+      <c r="L65" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M65" s="32"/>
       <c r="N65" s="32"/>
@@ -6205,7 +6358,7 @@
       <c r="B66" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C66" s="79" t="s">
+      <c r="C66" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D66" s="29" t="s">
@@ -6218,14 +6371,14 @@
       <c r="G66" s="31"/>
       <c r="H66" s="31"/>
       <c r="I66" s="36"/>
-      <c r="J66" s="82" t="s">
+      <c r="J66" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K66" s="82" t="s">
+      <c r="K66" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L66" s="82" t="s">
-        <v>634</v>
+      <c r="L66" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M66" s="32"/>
       <c r="N66" s="32"/>
@@ -6241,14 +6394,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="131.25" customHeight="1" thickBot="1">
+    <row r="67" spans="1:23" ht="18" customHeight="1" thickBot="1">
       <c r="A67" s="29">
         <v>92</v>
       </c>
       <c r="B67" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C67" s="79" t="s">
+      <c r="C67" s="101" t="s">
         <v>54</v>
       </c>
       <c r="D67" s="29" t="s">
@@ -6261,22 +6414,32 @@
       <c r="G67" s="31"/>
       <c r="H67" s="31"/>
       <c r="I67" s="36"/>
-      <c r="J67" s="82" t="s">
+      <c r="J67" s="80" t="s">
+        <v>75</v>
+      </c>
+      <c r="K67" s="80"/>
+      <c r="L67" s="80"/>
+      <c r="M67" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="N67" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="O67" s="100" t="s">
+        <v>648</v>
+      </c>
+      <c r="P67" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q67" s="100" t="s">
         <v>541</v>
       </c>
-      <c r="K67" s="82" t="s">
-        <v>505</v>
-      </c>
-      <c r="L67" s="82" t="s">
-        <v>634</v>
-      </c>
-      <c r="M67" s="32"/>
-      <c r="N67" s="32"/>
-      <c r="O67" s="32"/>
-      <c r="P67" s="32"/>
-      <c r="Q67" s="32"/>
-      <c r="R67" s="32"/>
-      <c r="S67" s="32"/>
+      <c r="R67" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="S67" s="84" t="s">
+        <v>639</v>
+      </c>
       <c r="T67" s="32"/>
       <c r="U67" s="33"/>
       <c r="V67" s="34"/>
@@ -6291,7 +6454,7 @@
       <c r="B68" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C68" s="79" t="s">
+      <c r="C68" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D68" s="29" t="s">
@@ -6307,7 +6470,7 @@
       <c r="J68" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K68" s="74"/>
+      <c r="K68" s="85"/>
       <c r="L68" s="32"/>
       <c r="M68" s="32"/>
       <c r="N68" s="32"/>
@@ -8208,7 +8371,7 @@
       <c r="J119" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K119" s="85" t="s">
+      <c r="K119" s="83" t="s">
         <v>503</v>
       </c>
       <c r="L119" s="32"/>
@@ -8233,7 +8396,7 @@
       <c r="B120" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C120" s="84" t="s">
+      <c r="C120" s="82" t="s">
         <v>56</v>
       </c>
       <c r="D120" s="29" t="s">
@@ -8249,7 +8412,7 @@
       <c r="J120" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K120" s="82" t="s">
+      <c r="K120" s="80" t="s">
         <v>504</v>
       </c>
       <c r="L120" s="32"/>
@@ -8274,7 +8437,7 @@
       <c r="B121" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C121" s="84" t="s">
+      <c r="C121" s="82" t="s">
         <v>56</v>
       </c>
       <c r="D121" s="29" t="s">
@@ -8290,7 +8453,7 @@
       <c r="J121" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K121" s="82" t="s">
+      <c r="K121" s="80" t="s">
         <v>500</v>
       </c>
       <c r="L121" s="32"/>
@@ -8315,7 +8478,7 @@
       <c r="B122" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C122" s="84" t="s">
+      <c r="C122" s="82" t="s">
         <v>56</v>
       </c>
       <c r="D122" s="29" t="s">
@@ -8356,7 +8519,7 @@
       <c r="B123" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C123" s="79" t="s">
+      <c r="C123" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D123" s="29" t="s">
@@ -8369,14 +8532,14 @@
       <c r="G123" s="31"/>
       <c r="H123" s="31"/>
       <c r="I123" s="36"/>
-      <c r="J123" s="82" t="s">
+      <c r="J123" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K123" s="82" t="s">
+      <c r="K123" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L123" s="82" t="s">
-        <v>634</v>
+      <c r="L123" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M123" s="32"/>
       <c r="N123" s="32"/>
@@ -8399,7 +8562,7 @@
       <c r="B124" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C124" s="79" t="s">
+      <c r="C124" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D124" s="29" t="s">
@@ -8412,14 +8575,14 @@
       <c r="G124" s="31"/>
       <c r="H124" s="31"/>
       <c r="I124" s="36"/>
-      <c r="J124" s="82" t="s">
+      <c r="J124" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K124" s="82" t="s">
+      <c r="K124" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L124" s="82" t="s">
-        <v>634</v>
+      <c r="L124" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M124" s="32"/>
       <c r="N124" s="32"/>
@@ -8442,7 +8605,7 @@
       <c r="B125" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C125" s="79" t="s">
+      <c r="C125" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D125" s="29" t="s">
@@ -8455,14 +8618,14 @@
       <c r="G125" s="31"/>
       <c r="H125" s="31"/>
       <c r="I125" s="36"/>
-      <c r="J125" s="82" t="s">
+      <c r="J125" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K125" s="82" t="s">
+      <c r="K125" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L125" s="82" t="s">
-        <v>634</v>
+      <c r="L125" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M125" s="32"/>
       <c r="N125" s="32"/>
@@ -8485,7 +8648,7 @@
       <c r="B126" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C126" s="79" t="s">
+      <c r="C126" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D126" s="29" t="s">
@@ -8498,14 +8661,14 @@
       <c r="G126" s="31"/>
       <c r="H126" s="31"/>
       <c r="I126" s="36"/>
-      <c r="J126" s="82" t="s">
+      <c r="J126" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K126" s="82" t="s">
+      <c r="K126" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L126" s="82" t="s">
-        <v>634</v>
+      <c r="L126" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M126" s="32"/>
       <c r="N126" s="32"/>
@@ -8528,7 +8691,7 @@
       <c r="B127" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C127" s="79" t="s">
+      <c r="C127" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D127" s="29" t="s">
@@ -8541,14 +8704,14 @@
       <c r="G127" s="31"/>
       <c r="H127" s="31"/>
       <c r="I127" s="36"/>
-      <c r="J127" s="82" t="s">
+      <c r="J127" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K127" s="82" t="s">
+      <c r="K127" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L127" s="82" t="s">
-        <v>634</v>
+      <c r="L127" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M127" s="32"/>
       <c r="N127" s="32"/>
@@ -8571,7 +8734,7 @@
       <c r="B128" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C128" s="79" t="s">
+      <c r="C128" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D128" s="29" t="s">
@@ -8584,14 +8747,14 @@
       <c r="G128" s="31"/>
       <c r="H128" s="31"/>
       <c r="I128" s="36"/>
-      <c r="J128" s="82" t="s">
+      <c r="J128" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K128" s="82" t="s">
+      <c r="K128" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L128" s="82" t="s">
-        <v>634</v>
+      <c r="L128" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M128" s="32"/>
       <c r="N128" s="32"/>
@@ -8614,7 +8777,7 @@
       <c r="B129" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C129" s="79" t="s">
+      <c r="C129" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D129" s="29" t="s">
@@ -8627,14 +8790,14 @@
       <c r="G129" s="31"/>
       <c r="H129" s="31"/>
       <c r="I129" s="36"/>
-      <c r="J129" s="82" t="s">
+      <c r="J129" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K129" s="82" t="s">
+      <c r="K129" s="80" t="s">
         <v>505</v>
       </c>
-      <c r="L129" s="82" t="s">
-        <v>634</v>
+      <c r="L129" s="80" t="s">
+        <v>633</v>
       </c>
       <c r="M129" s="32"/>
       <c r="N129" s="32"/>
@@ -8657,7 +8820,7 @@
       <c r="B130" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C130" s="79" t="s">
+      <c r="C130" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D130" s="29" t="s">
@@ -9910,14 +10073,14 @@
         <v>49</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="164" spans="1:23" ht="141.75" customHeight="1" thickBot="1">
       <c r="A164" s="29">
         <v>448</v>
       </c>
       <c r="B164" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C164" s="81" t="s">
+      <c r="C164" s="79" t="s">
         <v>56</v>
       </c>
       <c r="D164" s="29" t="s">
@@ -9926,11 +10089,19 @@
       <c r="E164" s="37" t="s">
         <v>341</v>
       </c>
-      <c r="F164" s="31"/>
+      <c r="F164" s="31">
+        <v>46143</v>
+      </c>
       <c r="G164" s="31"/>
-      <c r="H164" s="31"/>
-      <c r="I164" s="36"/>
-      <c r="J164" s="32"/>
+      <c r="H164" s="31" t="s">
+        <v>635</v>
+      </c>
+      <c r="I164" s="36" t="s">
+        <v>634</v>
+      </c>
+      <c r="J164" s="80" t="s">
+        <v>75</v>
+      </c>
       <c r="K164" s="32"/>
       <c r="L164" s="32"/>
       <c r="M164" s="32"/>
@@ -10358,7 +10529,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="176" spans="1:23" ht="165.75" customHeight="1" thickBot="1">
       <c r="A176" s="29">
         <v>461</v>
       </c>
@@ -10374,26 +10545,42 @@
       <c r="E176" s="37" t="s">
         <v>365</v>
       </c>
-      <c r="F176" s="29"/>
+      <c r="F176" s="98">
+        <v>46146</v>
+      </c>
       <c r="G176" s="29"/>
-      <c r="H176" s="29"/>
-      <c r="I176" s="29"/>
-      <c r="J176" s="82" t="s">
+      <c r="H176" s="29" t="s">
+        <v>645</v>
+      </c>
+      <c r="I176" s="29" t="s">
+        <v>646</v>
+      </c>
+      <c r="J176" s="80" t="s">
+        <v>75</v>
+      </c>
+      <c r="K176" s="80"/>
+      <c r="L176" s="80"/>
+      <c r="M176" s="99" t="s">
+        <v>75</v>
+      </c>
+      <c r="N176" s="99" t="s">
+        <v>75</v>
+      </c>
+      <c r="O176" s="99" t="s">
+        <v>647</v>
+      </c>
+      <c r="P176" s="99" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q176" s="99" t="s">
         <v>541</v>
       </c>
-      <c r="K176" s="82" t="s">
-        <v>505</v>
-      </c>
-      <c r="L176" s="82" t="s">
-        <v>634</v>
-      </c>
-      <c r="M176" s="32"/>
-      <c r="N176" s="32"/>
-      <c r="O176" s="29"/>
-      <c r="P176" s="32"/>
-      <c r="Q176" s="32"/>
-      <c r="R176" s="32"/>
-      <c r="S176" s="29"/>
+      <c r="R176" s="99" t="s">
+        <v>75</v>
+      </c>
+      <c r="S176" s="84" t="s">
+        <v>639</v>
+      </c>
       <c r="T176" s="32"/>
       <c r="U176" s="29"/>
       <c r="V176" s="29"/>
@@ -10408,7 +10595,7 @@
       <c r="B177" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C177" s="79" t="s">
+      <c r="C177" s="78" t="s">
         <v>54</v>
       </c>
       <c r="D177" s="29" t="s">
@@ -10424,8 +10611,8 @@
       <c r="J177" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K177" s="74" t="s">
-        <v>635</v>
+      <c r="K177" s="85" t="s">
+        <v>644</v>
       </c>
       <c r="L177" s="29"/>
       <c r="M177" s="32"/>
@@ -10627,7 +10814,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="16.5" customHeight="1" thickBot="1">
+    <row r="183" spans="1:23" ht="162" customHeight="1" thickBot="1">
       <c r="A183" s="29">
         <v>468</v>
       </c>
@@ -10647,11 +10834,11 @@
       <c r="G183" s="29"/>
       <c r="H183" s="29"/>
       <c r="I183" s="29"/>
-      <c r="J183" s="82" t="s">
+      <c r="J183" s="80" t="s">
         <v>541</v>
       </c>
       <c r="K183" s="85" t="s">
-        <v>503</v>
+        <v>644</v>
       </c>
       <c r="L183" s="29"/>
       <c r="M183" s="32"/>
@@ -10705,7 +10892,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="16.5" hidden="1" customHeight="1" thickBot="1">
+    <row r="185" spans="1:23" ht="140.25" hidden="1" customHeight="1" thickBot="1">
       <c r="A185" s="29">
         <v>470</v>
       </c>
@@ -10749,7 +10936,7 @@
       <c r="B186" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C186" s="80" t="s">
+      <c r="C186" s="78" t="s">
         <v>54</v>
       </c>
       <c r="D186" s="29" t="s">
@@ -10758,10 +10945,16 @@
       <c r="E186" s="37" t="s">
         <v>385</v>
       </c>
-      <c r="F186" s="31"/>
+      <c r="F186" s="31">
+        <v>46145</v>
+      </c>
       <c r="G186" s="31"/>
-      <c r="H186" s="31"/>
-      <c r="I186" s="36"/>
+      <c r="H186" s="31" t="s">
+        <v>636</v>
+      </c>
+      <c r="I186" s="36" t="s">
+        <v>637</v>
+      </c>
       <c r="J186" s="32" t="s">
         <v>75</v>
       </c>
@@ -10808,7 +11001,7 @@
         <v>505</v>
       </c>
       <c r="L187" s="32" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="M187" s="32"/>
       <c r="N187" s="32"/>
@@ -10870,7 +11063,7 @@
       <c r="B189" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C189" s="79" t="s">
+      <c r="C189" s="77" t="s">
         <v>54</v>
       </c>
       <c r="D189" s="29" t="s">
@@ -10886,7 +11079,7 @@
       <c r="J189" s="32" t="s">
         <v>541</v>
       </c>
-      <c r="K189" s="73" t="s">
+      <c r="K189" s="72" t="s">
         <v>503</v>
       </c>
       <c r="L189" s="32"/>
@@ -10911,7 +11104,7 @@
       <c r="B190" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="C190" s="79" t="s">
+      <c r="C190" s="77" t="s">
         <v>56</v>
       </c>
       <c r="D190" s="29" t="s">
@@ -10924,10 +11117,10 @@
       <c r="G190" s="31"/>
       <c r="H190" s="31"/>
       <c r="I190" s="36"/>
-      <c r="J190" s="82" t="s">
+      <c r="J190" s="80" t="s">
         <v>541</v>
       </c>
-      <c r="K190" s="85" t="s">
+      <c r="K190" s="83" t="s">
         <v>503</v>
       </c>
       <c r="L190" s="32"/>
@@ -16662,9 +16855,13 @@
     <mergeCell ref="C5:D5"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K53 K116 K165">
       <formula1>'[1]LISTA VALORI'!$A$2:$A$8</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M14:N15 P14:R15 M22:N23 P22:R23">
+      <formula1>[2]Sheet1!$B$2:$B$3</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>